<commit_message>
Sync plate designer: mixed sample type annotation
Mirrors NanoLlama/Phage_Display_Sequencing: sample type blocks in ordered
placement, composition in the Lab Plate Maps plate header, and per-well type
tags on mixed plates.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QBH1P2zpiSLx4BR7WKjhzK
</commit_message>
<xml_diff>
--- a/PhIPSeq_Manifest_Template_v4.xlsx
+++ b/PhIPSeq_Manifest_Template_v4.xlsx
@@ -618,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:D34"/>
+  <dimension ref="B2:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>96-well plate grids filled with input_id values. Shows physical plate layout.</t>
+          <t>96-well plate grids filled with input_id values. Shows physical plate layout. On plates carrying more than one sample type, the header names the composition and each well is tagged, e.g. SER-001 [serum].</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>96-well plate grids filled with tiu_id values. Used for downstream analysis.</t>
+          <t>96-well plate grids filled with tiu_id values. Used for downstream analysis — never annotated, so cells stay exact identifiers.</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -750,7 +750,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14"/>
     <row r="15">
       <c r="B15" s="9" t="inlineStr">
@@ -1014,7 +1013,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="B32" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sync plate designer: bridging samples, plate suffixes, control areas
Mirrors NanoLlama/Phage_Display_Sequencing.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QBH1P2zpiSLx4BR7WKjhzK
</commit_message>
<xml_diff>
--- a/PhIPSeq_Manifest_Template_v4.xlsx
+++ b/PhIPSeq_Manifest_Template_v4.xlsx
@@ -618,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D34"/>
+  <dimension ref="A2:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1013,32 +1013,50 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="9" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>repeat_across_plates</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Optional. Marks a bridging sample that runs on more than one plate (a highly reactive serum used as an anchor). Use "all" for every plate, or a list such as "1,3,5". Such samples get a -P1 / -P2 suffix in both plate map tabs.</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Color Legend</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="12" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>██</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Yellow cells = investigator fills in</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="13" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>██</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Blue italic row = example (delete before uploading)</t>
         </is>
@@ -1061,7 +1079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N102"/>
+  <dimension ref="A1:O102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1078,6 +1096,7 @@
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="28" customWidth="1" min="13" max="13"/>
     <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1151,6 +1170,11 @@
           <t>dither_group</t>
         </is>
       </c>
+      <c r="O1" s="14" t="inlineStr">
+        <is>
+          <t>repeat_across_plates</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
@@ -1213,6 +1237,7 @@
         </is>
       </c>
       <c r="N2" s="15" t="n"/>
+      <c r="O2" s="15" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="16" t="n"/>
@@ -1229,6 +1254,7 @@
       <c r="L3" s="16" t="n"/>
       <c r="M3" s="16" t="n"/>
       <c r="N3" s="16" t="n"/>
+      <c r="O3" s="16" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="16" t="n"/>
@@ -1245,6 +1271,7 @@
       <c r="L4" s="16" t="n"/>
       <c r="M4" s="16" t="n"/>
       <c r="N4" s="16" t="n"/>
+      <c r="O4" s="16" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="16" t="n"/>
@@ -1261,6 +1288,7 @@
       <c r="L5" s="16" t="n"/>
       <c r="M5" s="16" t="n"/>
       <c r="N5" s="16" t="n"/>
+      <c r="O5" s="16" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="16" t="n"/>
@@ -1277,6 +1305,7 @@
       <c r="L6" s="16" t="n"/>
       <c r="M6" s="16" t="n"/>
       <c r="N6" s="16" t="n"/>
+      <c r="O6" s="16" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="16" t="n"/>
@@ -1293,6 +1322,7 @@
       <c r="L7" s="16" t="n"/>
       <c r="M7" s="16" t="n"/>
       <c r="N7" s="16" t="n"/>
+      <c r="O7" s="16" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="16" t="n"/>
@@ -1309,6 +1339,7 @@
       <c r="L8" s="16" t="n"/>
       <c r="M8" s="16" t="n"/>
       <c r="N8" s="16" t="n"/>
+      <c r="O8" s="16" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="16" t="n"/>
@@ -1325,6 +1356,7 @@
       <c r="L9" s="16" t="n"/>
       <c r="M9" s="16" t="n"/>
       <c r="N9" s="16" t="n"/>
+      <c r="O9" s="16" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="16" t="n"/>
@@ -1341,6 +1373,7 @@
       <c r="L10" s="16" t="n"/>
       <c r="M10" s="16" t="n"/>
       <c r="N10" s="16" t="n"/>
+      <c r="O10" s="16" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="16" t="n"/>
@@ -1357,6 +1390,7 @@
       <c r="L11" s="16" t="n"/>
       <c r="M11" s="16" t="n"/>
       <c r="N11" s="16" t="n"/>
+      <c r="O11" s="16" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="16" t="n"/>
@@ -1373,6 +1407,7 @@
       <c r="L12" s="16" t="n"/>
       <c r="M12" s="16" t="n"/>
       <c r="N12" s="16" t="n"/>
+      <c r="O12" s="16" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="16" t="n"/>
@@ -1389,6 +1424,7 @@
       <c r="L13" s="16" t="n"/>
       <c r="M13" s="16" t="n"/>
       <c r="N13" s="16" t="n"/>
+      <c r="O13" s="16" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="16" t="n"/>
@@ -1405,6 +1441,7 @@
       <c r="L14" s="16" t="n"/>
       <c r="M14" s="16" t="n"/>
       <c r="N14" s="16" t="n"/>
+      <c r="O14" s="16" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="16" t="n"/>
@@ -1421,6 +1458,7 @@
       <c r="L15" s="16" t="n"/>
       <c r="M15" s="16" t="n"/>
       <c r="N15" s="16" t="n"/>
+      <c r="O15" s="16" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="16" t="n"/>
@@ -1437,6 +1475,7 @@
       <c r="L16" s="16" t="n"/>
       <c r="M16" s="16" t="n"/>
       <c r="N16" s="16" t="n"/>
+      <c r="O16" s="16" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="16" t="n"/>
@@ -1453,6 +1492,7 @@
       <c r="L17" s="16" t="n"/>
       <c r="M17" s="16" t="n"/>
       <c r="N17" s="16" t="n"/>
+      <c r="O17" s="16" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="16" t="n"/>
@@ -1469,6 +1509,7 @@
       <c r="L18" s="16" t="n"/>
       <c r="M18" s="16" t="n"/>
       <c r="N18" s="16" t="n"/>
+      <c r="O18" s="16" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="16" t="n"/>
@@ -1485,6 +1526,7 @@
       <c r="L19" s="16" t="n"/>
       <c r="M19" s="16" t="n"/>
       <c r="N19" s="16" t="n"/>
+      <c r="O19" s="16" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="16" t="n"/>
@@ -1501,6 +1543,7 @@
       <c r="L20" s="16" t="n"/>
       <c r="M20" s="16" t="n"/>
       <c r="N20" s="16" t="n"/>
+      <c r="O20" s="16" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="16" t="n"/>
@@ -1517,6 +1560,7 @@
       <c r="L21" s="16" t="n"/>
       <c r="M21" s="16" t="n"/>
       <c r="N21" s="16" t="n"/>
+      <c r="O21" s="16" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="16" t="n"/>
@@ -1533,6 +1577,7 @@
       <c r="L22" s="16" t="n"/>
       <c r="M22" s="16" t="n"/>
       <c r="N22" s="16" t="n"/>
+      <c r="O22" s="16" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="16" t="n"/>
@@ -1549,6 +1594,7 @@
       <c r="L23" s="16" t="n"/>
       <c r="M23" s="16" t="n"/>
       <c r="N23" s="16" t="n"/>
+      <c r="O23" s="16" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="16" t="n"/>
@@ -1565,6 +1611,7 @@
       <c r="L24" s="16" t="n"/>
       <c r="M24" s="16" t="n"/>
       <c r="N24" s="16" t="n"/>
+      <c r="O24" s="16" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="16" t="n"/>
@@ -1581,6 +1628,7 @@
       <c r="L25" s="16" t="n"/>
       <c r="M25" s="16" t="n"/>
       <c r="N25" s="16" t="n"/>
+      <c r="O25" s="16" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="16" t="n"/>
@@ -1597,6 +1645,7 @@
       <c r="L26" s="16" t="n"/>
       <c r="M26" s="16" t="n"/>
       <c r="N26" s="16" t="n"/>
+      <c r="O26" s="16" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="16" t="n"/>
@@ -1613,6 +1662,7 @@
       <c r="L27" s="16" t="n"/>
       <c r="M27" s="16" t="n"/>
       <c r="N27" s="16" t="n"/>
+      <c r="O27" s="16" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="16" t="n"/>
@@ -1629,6 +1679,7 @@
       <c r="L28" s="16" t="n"/>
       <c r="M28" s="16" t="n"/>
       <c r="N28" s="16" t="n"/>
+      <c r="O28" s="16" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="16" t="n"/>
@@ -1645,6 +1696,7 @@
       <c r="L29" s="16" t="n"/>
       <c r="M29" s="16" t="n"/>
       <c r="N29" s="16" t="n"/>
+      <c r="O29" s="16" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="16" t="n"/>
@@ -1661,6 +1713,7 @@
       <c r="L30" s="16" t="n"/>
       <c r="M30" s="16" t="n"/>
       <c r="N30" s="16" t="n"/>
+      <c r="O30" s="16" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="16" t="n"/>
@@ -1677,6 +1730,7 @@
       <c r="L31" s="16" t="n"/>
       <c r="M31" s="16" t="n"/>
       <c r="N31" s="16" t="n"/>
+      <c r="O31" s="16" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="16" t="n"/>
@@ -1693,6 +1747,7 @@
       <c r="L32" s="16" t="n"/>
       <c r="M32" s="16" t="n"/>
       <c r="N32" s="16" t="n"/>
+      <c r="O32" s="16" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="16" t="n"/>
@@ -1709,6 +1764,7 @@
       <c r="L33" s="16" t="n"/>
       <c r="M33" s="16" t="n"/>
       <c r="N33" s="16" t="n"/>
+      <c r="O33" s="16" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="16" t="n"/>
@@ -1725,6 +1781,7 @@
       <c r="L34" s="16" t="n"/>
       <c r="M34" s="16" t="n"/>
       <c r="N34" s="16" t="n"/>
+      <c r="O34" s="16" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="16" t="n"/>
@@ -1741,6 +1798,7 @@
       <c r="L35" s="16" t="n"/>
       <c r="M35" s="16" t="n"/>
       <c r="N35" s="16" t="n"/>
+      <c r="O35" s="16" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="16" t="n"/>
@@ -1757,6 +1815,7 @@
       <c r="L36" s="16" t="n"/>
       <c r="M36" s="16" t="n"/>
       <c r="N36" s="16" t="n"/>
+      <c r="O36" s="16" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="16" t="n"/>
@@ -1773,6 +1832,7 @@
       <c r="L37" s="16" t="n"/>
       <c r="M37" s="16" t="n"/>
       <c r="N37" s="16" t="n"/>
+      <c r="O37" s="16" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="16" t="n"/>
@@ -1789,6 +1849,7 @@
       <c r="L38" s="16" t="n"/>
       <c r="M38" s="16" t="n"/>
       <c r="N38" s="16" t="n"/>
+      <c r="O38" s="16" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="16" t="n"/>
@@ -1805,6 +1866,7 @@
       <c r="L39" s="16" t="n"/>
       <c r="M39" s="16" t="n"/>
       <c r="N39" s="16" t="n"/>
+      <c r="O39" s="16" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="16" t="n"/>
@@ -1821,6 +1883,7 @@
       <c r="L40" s="16" t="n"/>
       <c r="M40" s="16" t="n"/>
       <c r="N40" s="16" t="n"/>
+      <c r="O40" s="16" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="16" t="n"/>
@@ -1837,6 +1900,7 @@
       <c r="L41" s="16" t="n"/>
       <c r="M41" s="16" t="n"/>
       <c r="N41" s="16" t="n"/>
+      <c r="O41" s="16" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="16" t="n"/>
@@ -1853,6 +1917,7 @@
       <c r="L42" s="16" t="n"/>
       <c r="M42" s="16" t="n"/>
       <c r="N42" s="16" t="n"/>
+      <c r="O42" s="16" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="16" t="n"/>
@@ -1869,6 +1934,7 @@
       <c r="L43" s="16" t="n"/>
       <c r="M43" s="16" t="n"/>
       <c r="N43" s="16" t="n"/>
+      <c r="O43" s="16" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="16" t="n"/>
@@ -1885,6 +1951,7 @@
       <c r="L44" s="16" t="n"/>
       <c r="M44" s="16" t="n"/>
       <c r="N44" s="16" t="n"/>
+      <c r="O44" s="16" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="16" t="n"/>
@@ -1901,6 +1968,7 @@
       <c r="L45" s="16" t="n"/>
       <c r="M45" s="16" t="n"/>
       <c r="N45" s="16" t="n"/>
+      <c r="O45" s="16" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="16" t="n"/>
@@ -1917,6 +1985,7 @@
       <c r="L46" s="16" t="n"/>
       <c r="M46" s="16" t="n"/>
       <c r="N46" s="16" t="n"/>
+      <c r="O46" s="16" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="16" t="n"/>
@@ -1933,6 +2002,7 @@
       <c r="L47" s="16" t="n"/>
       <c r="M47" s="16" t="n"/>
       <c r="N47" s="16" t="n"/>
+      <c r="O47" s="16" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="16" t="n"/>
@@ -1949,6 +2019,7 @@
       <c r="L48" s="16" t="n"/>
       <c r="M48" s="16" t="n"/>
       <c r="N48" s="16" t="n"/>
+      <c r="O48" s="16" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="16" t="n"/>
@@ -1965,6 +2036,7 @@
       <c r="L49" s="16" t="n"/>
       <c r="M49" s="16" t="n"/>
       <c r="N49" s="16" t="n"/>
+      <c r="O49" s="16" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="16" t="n"/>
@@ -1981,6 +2053,7 @@
       <c r="L50" s="16" t="n"/>
       <c r="M50" s="16" t="n"/>
       <c r="N50" s="16" t="n"/>
+      <c r="O50" s="16" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="16" t="n"/>
@@ -1997,6 +2070,7 @@
       <c r="L51" s="16" t="n"/>
       <c r="M51" s="16" t="n"/>
       <c r="N51" s="16" t="n"/>
+      <c r="O51" s="16" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="16" t="n"/>
@@ -2013,6 +2087,7 @@
       <c r="L52" s="16" t="n"/>
       <c r="M52" s="16" t="n"/>
       <c r="N52" s="16" t="n"/>
+      <c r="O52" s="16" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="16" t="n"/>
@@ -2029,6 +2104,7 @@
       <c r="L53" s="16" t="n"/>
       <c r="M53" s="16" t="n"/>
       <c r="N53" s="16" t="n"/>
+      <c r="O53" s="16" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="16" t="n"/>
@@ -2045,6 +2121,7 @@
       <c r="L54" s="16" t="n"/>
       <c r="M54" s="16" t="n"/>
       <c r="N54" s="16" t="n"/>
+      <c r="O54" s="16" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="16" t="n"/>
@@ -2061,6 +2138,7 @@
       <c r="L55" s="16" t="n"/>
       <c r="M55" s="16" t="n"/>
       <c r="N55" s="16" t="n"/>
+      <c r="O55" s="16" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="n"/>
@@ -2077,6 +2155,7 @@
       <c r="L56" s="16" t="n"/>
       <c r="M56" s="16" t="n"/>
       <c r="N56" s="16" t="n"/>
+      <c r="O56" s="16" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="16" t="n"/>
@@ -2093,6 +2172,7 @@
       <c r="L57" s="16" t="n"/>
       <c r="M57" s="16" t="n"/>
       <c r="N57" s="16" t="n"/>
+      <c r="O57" s="16" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="16" t="n"/>
@@ -2109,6 +2189,7 @@
       <c r="L58" s="16" t="n"/>
       <c r="M58" s="16" t="n"/>
       <c r="N58" s="16" t="n"/>
+      <c r="O58" s="16" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="16" t="n"/>
@@ -2125,6 +2206,7 @@
       <c r="L59" s="16" t="n"/>
       <c r="M59" s="16" t="n"/>
       <c r="N59" s="16" t="n"/>
+      <c r="O59" s="16" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="16" t="n"/>
@@ -2141,6 +2223,7 @@
       <c r="L60" s="16" t="n"/>
       <c r="M60" s="16" t="n"/>
       <c r="N60" s="16" t="n"/>
+      <c r="O60" s="16" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="16" t="n"/>
@@ -2157,6 +2240,7 @@
       <c r="L61" s="16" t="n"/>
       <c r="M61" s="16" t="n"/>
       <c r="N61" s="16" t="n"/>
+      <c r="O61" s="16" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="16" t="n"/>
@@ -2173,6 +2257,7 @@
       <c r="L62" s="16" t="n"/>
       <c r="M62" s="16" t="n"/>
       <c r="N62" s="16" t="n"/>
+      <c r="O62" s="16" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="16" t="n"/>
@@ -2189,6 +2274,7 @@
       <c r="L63" s="16" t="n"/>
       <c r="M63" s="16" t="n"/>
       <c r="N63" s="16" t="n"/>
+      <c r="O63" s="16" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="16" t="n"/>
@@ -2205,6 +2291,7 @@
       <c r="L64" s="16" t="n"/>
       <c r="M64" s="16" t="n"/>
       <c r="N64" s="16" t="n"/>
+      <c r="O64" s="16" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="16" t="n"/>
@@ -2221,6 +2308,7 @@
       <c r="L65" s="16" t="n"/>
       <c r="M65" s="16" t="n"/>
       <c r="N65" s="16" t="n"/>
+      <c r="O65" s="16" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="16" t="n"/>
@@ -2237,6 +2325,7 @@
       <c r="L66" s="16" t="n"/>
       <c r="M66" s="16" t="n"/>
       <c r="N66" s="16" t="n"/>
+      <c r="O66" s="16" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="16" t="n"/>
@@ -2253,6 +2342,7 @@
       <c r="L67" s="16" t="n"/>
       <c r="M67" s="16" t="n"/>
       <c r="N67" s="16" t="n"/>
+      <c r="O67" s="16" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="16" t="n"/>
@@ -2269,6 +2359,7 @@
       <c r="L68" s="16" t="n"/>
       <c r="M68" s="16" t="n"/>
       <c r="N68" s="16" t="n"/>
+      <c r="O68" s="16" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="16" t="n"/>
@@ -2285,6 +2376,7 @@
       <c r="L69" s="16" t="n"/>
       <c r="M69" s="16" t="n"/>
       <c r="N69" s="16" t="n"/>
+      <c r="O69" s="16" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="16" t="n"/>
@@ -2301,6 +2393,7 @@
       <c r="L70" s="16" t="n"/>
       <c r="M70" s="16" t="n"/>
       <c r="N70" s="16" t="n"/>
+      <c r="O70" s="16" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="16" t="n"/>
@@ -2317,6 +2410,7 @@
       <c r="L71" s="16" t="n"/>
       <c r="M71" s="16" t="n"/>
       <c r="N71" s="16" t="n"/>
+      <c r="O71" s="16" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="16" t="n"/>
@@ -2333,6 +2427,7 @@
       <c r="L72" s="16" t="n"/>
       <c r="M72" s="16" t="n"/>
       <c r="N72" s="16" t="n"/>
+      <c r="O72" s="16" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="16" t="n"/>
@@ -2349,6 +2444,7 @@
       <c r="L73" s="16" t="n"/>
       <c r="M73" s="16" t="n"/>
       <c r="N73" s="16" t="n"/>
+      <c r="O73" s="16" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="16" t="n"/>
@@ -2365,6 +2461,7 @@
       <c r="L74" s="16" t="n"/>
       <c r="M74" s="16" t="n"/>
       <c r="N74" s="16" t="n"/>
+      <c r="O74" s="16" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="16" t="n"/>
@@ -2381,6 +2478,7 @@
       <c r="L75" s="16" t="n"/>
       <c r="M75" s="16" t="n"/>
       <c r="N75" s="16" t="n"/>
+      <c r="O75" s="16" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="16" t="n"/>
@@ -2397,6 +2495,7 @@
       <c r="L76" s="16" t="n"/>
       <c r="M76" s="16" t="n"/>
       <c r="N76" s="16" t="n"/>
+      <c r="O76" s="16" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="16" t="n"/>
@@ -2413,6 +2512,7 @@
       <c r="L77" s="16" t="n"/>
       <c r="M77" s="16" t="n"/>
       <c r="N77" s="16" t="n"/>
+      <c r="O77" s="16" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="16" t="n"/>
@@ -2429,6 +2529,7 @@
       <c r="L78" s="16" t="n"/>
       <c r="M78" s="16" t="n"/>
       <c r="N78" s="16" t="n"/>
+      <c r="O78" s="16" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="16" t="n"/>
@@ -2445,6 +2546,7 @@
       <c r="L79" s="16" t="n"/>
       <c r="M79" s="16" t="n"/>
       <c r="N79" s="16" t="n"/>
+      <c r="O79" s="16" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="16" t="n"/>
@@ -2461,6 +2563,7 @@
       <c r="L80" s="16" t="n"/>
       <c r="M80" s="16" t="n"/>
       <c r="N80" s="16" t="n"/>
+      <c r="O80" s="16" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="16" t="n"/>
@@ -2477,6 +2580,7 @@
       <c r="L81" s="16" t="n"/>
       <c r="M81" s="16" t="n"/>
       <c r="N81" s="16" t="n"/>
+      <c r="O81" s="16" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="16" t="n"/>
@@ -2493,6 +2597,7 @@
       <c r="L82" s="16" t="n"/>
       <c r="M82" s="16" t="n"/>
       <c r="N82" s="16" t="n"/>
+      <c r="O82" s="16" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="16" t="n"/>
@@ -2509,6 +2614,7 @@
       <c r="L83" s="16" t="n"/>
       <c r="M83" s="16" t="n"/>
       <c r="N83" s="16" t="n"/>
+      <c r="O83" s="16" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="16" t="n"/>
@@ -2525,6 +2631,7 @@
       <c r="L84" s="16" t="n"/>
       <c r="M84" s="16" t="n"/>
       <c r="N84" s="16" t="n"/>
+      <c r="O84" s="16" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="16" t="n"/>
@@ -2541,6 +2648,7 @@
       <c r="L85" s="16" t="n"/>
       <c r="M85" s="16" t="n"/>
       <c r="N85" s="16" t="n"/>
+      <c r="O85" s="16" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="16" t="n"/>
@@ -2557,6 +2665,7 @@
       <c r="L86" s="16" t="n"/>
       <c r="M86" s="16" t="n"/>
       <c r="N86" s="16" t="n"/>
+      <c r="O86" s="16" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="16" t="n"/>
@@ -2573,6 +2682,7 @@
       <c r="L87" s="16" t="n"/>
       <c r="M87" s="16" t="n"/>
       <c r="N87" s="16" t="n"/>
+      <c r="O87" s="16" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="16" t="n"/>
@@ -2589,6 +2699,7 @@
       <c r="L88" s="16" t="n"/>
       <c r="M88" s="16" t="n"/>
       <c r="N88" s="16" t="n"/>
+      <c r="O88" s="16" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="16" t="n"/>
@@ -2605,6 +2716,7 @@
       <c r="L89" s="16" t="n"/>
       <c r="M89" s="16" t="n"/>
       <c r="N89" s="16" t="n"/>
+      <c r="O89" s="16" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="16" t="n"/>
@@ -2621,6 +2733,7 @@
       <c r="L90" s="16" t="n"/>
       <c r="M90" s="16" t="n"/>
       <c r="N90" s="16" t="n"/>
+      <c r="O90" s="16" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="16" t="n"/>
@@ -2637,6 +2750,7 @@
       <c r="L91" s="16" t="n"/>
       <c r="M91" s="16" t="n"/>
       <c r="N91" s="16" t="n"/>
+      <c r="O91" s="16" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="16" t="n"/>
@@ -2653,6 +2767,7 @@
       <c r="L92" s="16" t="n"/>
       <c r="M92" s="16" t="n"/>
       <c r="N92" s="16" t="n"/>
+      <c r="O92" s="16" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="16" t="n"/>
@@ -2669,6 +2784,7 @@
       <c r="L93" s="16" t="n"/>
       <c r="M93" s="16" t="n"/>
       <c r="N93" s="16" t="n"/>
+      <c r="O93" s="16" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="16" t="n"/>
@@ -2685,6 +2801,7 @@
       <c r="L94" s="16" t="n"/>
       <c r="M94" s="16" t="n"/>
       <c r="N94" s="16" t="n"/>
+      <c r="O94" s="16" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="16" t="n"/>
@@ -2701,6 +2818,7 @@
       <c r="L95" s="16" t="n"/>
       <c r="M95" s="16" t="n"/>
       <c r="N95" s="16" t="n"/>
+      <c r="O95" s="16" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="16" t="n"/>
@@ -2717,6 +2835,7 @@
       <c r="L96" s="16" t="n"/>
       <c r="M96" s="16" t="n"/>
       <c r="N96" s="16" t="n"/>
+      <c r="O96" s="16" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="16" t="n"/>
@@ -2733,6 +2852,7 @@
       <c r="L97" s="16" t="n"/>
       <c r="M97" s="16" t="n"/>
       <c r="N97" s="16" t="n"/>
+      <c r="O97" s="16" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="16" t="n"/>
@@ -2749,6 +2869,7 @@
       <c r="L98" s="16" t="n"/>
       <c r="M98" s="16" t="n"/>
       <c r="N98" s="16" t="n"/>
+      <c r="O98" s="16" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="16" t="n"/>
@@ -2765,6 +2886,7 @@
       <c r="L99" s="16" t="n"/>
       <c r="M99" s="16" t="n"/>
       <c r="N99" s="16" t="n"/>
+      <c r="O99" s="16" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="16" t="n"/>
@@ -2781,6 +2903,7 @@
       <c r="L100" s="16" t="n"/>
       <c r="M100" s="16" t="n"/>
       <c r="N100" s="16" t="n"/>
+      <c r="O100" s="16" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="16" t="n"/>
@@ -2797,6 +2920,7 @@
       <c r="L101" s="16" t="n"/>
       <c r="M101" s="16" t="n"/>
       <c r="N101" s="16" t="n"/>
+      <c r="O101" s="16" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="16" t="n"/>
@@ -2813,6 +2937,7 @@
       <c r="L102" s="16" t="n"/>
       <c r="M102" s="16" t="n"/>
       <c r="N102" s="16" t="n"/>
+      <c r="O102" s="16" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M1"/>

</xml_diff>